<commit_message>
Speiseplan September 2026: korrigierte Zeiten (07.00 Uhr)
Katrins Fußzeile nannte noch 08.00 Uhr fuer Ab- und Bestellungen.
Neue Quelldatei mit 07.00 Uhr uebernommen (Bild, PDF, xlsx neu erzeugt).
Gerichte unveraendert -- DB und Chatbot brauchen keinen Reimport.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/speiseplan/2026-09-speiseplan-markersdorf.xlsx
+++ b/assets/speiseplan/2026-09-speiseplan-markersdorf.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr/>
   <bookViews>
     <workbookView xWindow="480" yWindow="120" windowWidth="8055" windowHeight="5895"/>
@@ -11,7 +11,7 @@
     <sheet name="Tabelle2" sheetId="2" r:id="rId2"/>
     <sheet name="Tabelle3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="125725"/>
 </workbook>
 </file>
 
@@ -118,6 +118,237 @@
   </si>
   <si>
     <t>Kartoffelbrei</t>
+  </si>
+  <si>
+    <t>Nudeln</t>
+  </si>
+  <si>
+    <t>Wurstgulasch</t>
+  </si>
+  <si>
+    <t>Kochklops</t>
+  </si>
+  <si>
+    <t>1.Kürbissuppe</t>
+  </si>
+  <si>
+    <t>mit Croutons</t>
+  </si>
+  <si>
+    <t>Omas Kartoffelsuppe</t>
+  </si>
+  <si>
+    <t>Nudelsuppe</t>
+  </si>
+  <si>
+    <t>Erbseneintopf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">und </t>
+  </si>
+  <si>
+    <t>Ei</t>
+  </si>
+  <si>
+    <t>7.9.</t>
+  </si>
+  <si>
+    <t>Spinat</t>
+  </si>
+  <si>
+    <t>Rindergulasch</t>
+  </si>
+  <si>
+    <t>Rotkraut</t>
+  </si>
+  <si>
+    <t>11.9.</t>
+  </si>
+  <si>
+    <t>Jägerschnitzel</t>
+  </si>
+  <si>
+    <t>Gemüse</t>
+  </si>
+  <si>
+    <t>14.9.</t>
+  </si>
+  <si>
+    <t>18.9.</t>
+  </si>
+  <si>
+    <t>21.9.</t>
+  </si>
+  <si>
+    <t>25.9.</t>
+  </si>
+  <si>
+    <t>28.9.</t>
+  </si>
+  <si>
+    <t>02.10.</t>
+  </si>
+  <si>
+    <t>2.Kohlrabieintopf</t>
+  </si>
+  <si>
+    <t>Mischgemüse</t>
+  </si>
+  <si>
+    <t>Kartoffeln</t>
+  </si>
+  <si>
+    <t>Carbonara</t>
+  </si>
+  <si>
+    <t>gedünsteter Fisch</t>
+  </si>
+  <si>
+    <t>Dillsoße</t>
+  </si>
+  <si>
+    <t>1.Milchreis,Kirschen</t>
+  </si>
+  <si>
+    <t>und Zimtzucker</t>
+  </si>
+  <si>
+    <t>2.Feuerfleisch</t>
+  </si>
+  <si>
+    <t>und Langkornreis</t>
+  </si>
+  <si>
+    <t>Blumenkohl</t>
+  </si>
+  <si>
+    <t>mit feinem</t>
+  </si>
+  <si>
+    <t>dazu Rote Bete</t>
+  </si>
+  <si>
+    <t>und Kräutersoße</t>
+  </si>
+  <si>
+    <t>Wildheidelbeeren</t>
+  </si>
+  <si>
+    <t>1.Hefeklöße,Vanillesoße</t>
+  </si>
+  <si>
+    <t>2.Bauernfrühstück</t>
+  </si>
+  <si>
+    <t>bunter Salat</t>
+  </si>
+  <si>
+    <t>Paprikasoße</t>
+  </si>
+  <si>
+    <t>Rahmgeschnetzeltes</t>
+  </si>
+  <si>
+    <t>Knöpfle</t>
+  </si>
+  <si>
+    <t>Brokkoli</t>
+  </si>
+  <si>
+    <t>Klöße</t>
+  </si>
+  <si>
+    <t>1.Reibekuchen mit</t>
+  </si>
+  <si>
+    <t>Apfelmus</t>
+  </si>
+  <si>
+    <t>2.Gulaschsuppe</t>
+  </si>
+  <si>
+    <t>Brötchen</t>
+  </si>
+  <si>
+    <t>1.Buttermilchplinse</t>
+  </si>
+  <si>
+    <t>Mango-Fruchtmus</t>
+  </si>
+  <si>
+    <t>2.Gyros,Zaziki</t>
+  </si>
+  <si>
+    <t>und Kartoffelspalten</t>
+  </si>
+  <si>
+    <t>Emmas Wunsch</t>
+  </si>
+  <si>
+    <t>gebratenes Hähnchen</t>
+  </si>
+  <si>
+    <t>Svens Wunsch</t>
+  </si>
+  <si>
+    <t>Risibisi</t>
+  </si>
+  <si>
+    <t>Werk 1 Wunsch</t>
+  </si>
+  <si>
+    <t>Schnitzel Wiener Art</t>
+  </si>
+  <si>
+    <t>Hannahs Wunsch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spaghetti </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kartoffeln </t>
+  </si>
+  <si>
+    <t>Fischstäbchen</t>
+  </si>
+  <si>
+    <t>Alfreds Wunsch</t>
+  </si>
+  <si>
+    <t>Paprika-Tomatensoße</t>
+  </si>
+  <si>
+    <t>und Zucchini /Reibekäse</t>
+  </si>
+  <si>
+    <t>Lewins Wunsch</t>
+  </si>
+  <si>
+    <t>Alinas Wunsch</t>
+  </si>
+  <si>
+    <t>Cheyennes Wunsch</t>
+  </si>
+  <si>
+    <t>Speiseplan September 2026 Schulküche Markersdorf</t>
+  </si>
+  <si>
+    <t>Bitte bis 31.08.26 in der App bestellen</t>
+  </si>
+  <si>
+    <t>Gemüse Couscous</t>
+  </si>
+  <si>
+    <t>Woche vom 7.9.-11.9.2026</t>
+  </si>
+  <si>
+    <t>Woche vom 14.9.-18.9.2026</t>
+  </si>
+  <si>
+    <t>Woche vom 21.9.-25.9.2026</t>
+  </si>
+  <si>
+    <t>Woche vom 28.9.-2.10.2026</t>
   </si>
   <si>
     <r>
@@ -139,7 +370,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> täglich bitte bis 08.00 Uhr, sonst müssen wir die Tage berechnen</t>
+      <t xml:space="preserve"> täglich bitte bis 07.00 Uhr, sonst müssen wir die Tage berechnen</t>
     </r>
   </si>
   <si>
@@ -162,239 +393,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> nehmen wir ebenfalls bis 08.00 Uhr entgegen</t>
+      <t xml:space="preserve"> nehmen wir ebenfalls bis 07.00 Uhr entgegen</t>
     </r>
-  </si>
-  <si>
-    <t>Nudeln</t>
-  </si>
-  <si>
-    <t>Wurstgulasch</t>
-  </si>
-  <si>
-    <t>Kochklops</t>
-  </si>
-  <si>
-    <t>1.Kürbissuppe</t>
-  </si>
-  <si>
-    <t>mit Croutons</t>
-  </si>
-  <si>
-    <t>Omas Kartoffelsuppe</t>
-  </si>
-  <si>
-    <t>Nudelsuppe</t>
-  </si>
-  <si>
-    <t>Erbseneintopf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">und </t>
-  </si>
-  <si>
-    <t>Ei</t>
-  </si>
-  <si>
-    <t>7.9.</t>
-  </si>
-  <si>
-    <t>Spinat</t>
-  </si>
-  <si>
-    <t>Rindergulasch</t>
-  </si>
-  <si>
-    <t>Rotkraut</t>
-  </si>
-  <si>
-    <t>11.9.</t>
-  </si>
-  <si>
-    <t>Jägerschnitzel</t>
-  </si>
-  <si>
-    <t>Gemüse</t>
-  </si>
-  <si>
-    <t>14.9.</t>
-  </si>
-  <si>
-    <t>18.9.</t>
-  </si>
-  <si>
-    <t>21.9.</t>
-  </si>
-  <si>
-    <t>25.9.</t>
-  </si>
-  <si>
-    <t>28.9.</t>
-  </si>
-  <si>
-    <t>02.10.</t>
-  </si>
-  <si>
-    <t>2.Kohlrabieintopf</t>
-  </si>
-  <si>
-    <t>Mischgemüse</t>
-  </si>
-  <si>
-    <t>Kartoffeln</t>
-  </si>
-  <si>
-    <t>Carbonara</t>
-  </si>
-  <si>
-    <t>gedünsteter Fisch</t>
-  </si>
-  <si>
-    <t>Dillsoße</t>
-  </si>
-  <si>
-    <t>1.Milchreis,Kirschen</t>
-  </si>
-  <si>
-    <t>und Zimtzucker</t>
-  </si>
-  <si>
-    <t>2.Feuerfleisch</t>
-  </si>
-  <si>
-    <t>und Langkornreis</t>
-  </si>
-  <si>
-    <t>Blumenkohl</t>
-  </si>
-  <si>
-    <t>mit feinem</t>
-  </si>
-  <si>
-    <t>dazu Rote Bete</t>
-  </si>
-  <si>
-    <t>und Kräutersoße</t>
-  </si>
-  <si>
-    <t>Wildheidelbeeren</t>
-  </si>
-  <si>
-    <t>1.Hefeklöße,Vanillesoße</t>
-  </si>
-  <si>
-    <t>2.Bauernfrühstück</t>
-  </si>
-  <si>
-    <t>bunter Salat</t>
-  </si>
-  <si>
-    <t>Paprikasoße</t>
-  </si>
-  <si>
-    <t>Rahmgeschnetzeltes</t>
-  </si>
-  <si>
-    <t>Knöpfle</t>
-  </si>
-  <si>
-    <t>Brokkoli</t>
-  </si>
-  <si>
-    <t>Klöße</t>
-  </si>
-  <si>
-    <t>1.Reibekuchen mit</t>
-  </si>
-  <si>
-    <t>Apfelmus</t>
-  </si>
-  <si>
-    <t>2.Gulaschsuppe</t>
-  </si>
-  <si>
-    <t>Brötchen</t>
-  </si>
-  <si>
-    <t>1.Buttermilchplinse</t>
-  </si>
-  <si>
-    <t>Mango-Fruchtmus</t>
-  </si>
-  <si>
-    <t>2.Gyros,Zaziki</t>
-  </si>
-  <si>
-    <t>und Kartoffelspalten</t>
-  </si>
-  <si>
-    <t>Emmas Wunsch</t>
-  </si>
-  <si>
-    <t>gebratenes Hähnchen</t>
-  </si>
-  <si>
-    <t>Svens Wunsch</t>
-  </si>
-  <si>
-    <t>Risibisi</t>
-  </si>
-  <si>
-    <t>Werk 1 Wunsch</t>
-  </si>
-  <si>
-    <t>Schnitzel Wiener Art</t>
-  </si>
-  <si>
-    <t>Hannahs Wunsch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spaghetti </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kartoffeln </t>
-  </si>
-  <si>
-    <t>Fischstäbchen</t>
-  </si>
-  <si>
-    <t>Alfreds Wunsch</t>
-  </si>
-  <si>
-    <t>Paprika-Tomatensoße</t>
-  </si>
-  <si>
-    <t>und Zucchini /Reibekäse</t>
-  </si>
-  <si>
-    <t>Lewins Wunsch</t>
-  </si>
-  <si>
-    <t>Alinas Wunsch</t>
-  </si>
-  <si>
-    <t>Cheyennes Wunsch</t>
-  </si>
-  <si>
-    <t>Speiseplan September 2026 Schulküche Markersdorf</t>
-  </si>
-  <si>
-    <t>Bitte bis 31.08.26 in der App bestellen</t>
-  </si>
-  <si>
-    <t>Gemüse Couscous</t>
-  </si>
-  <si>
-    <t>Woche vom 7.9.-11.9.2026</t>
-  </si>
-  <si>
-    <t>Woche vom 14.9.-18.9.2026</t>
-  </si>
-  <si>
-    <t>Woche vom 21.9.-25.9.2026</t>
-  </si>
-  <si>
-    <t>Woche vom 28.9.-2.10.2026</t>
   </si>
 </sst>
 </file>
@@ -977,24 +977,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="8" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1037,6 +1019,24 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1275,7 +1275,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
         <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
@@ -1706,23 +1706,23 @@
     <col min="7" max="12" width="3.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="30" thickBot="1">
+    <row r="1" spans="1:15" ht="24" thickBot="1">
       <c r="A1" s="1"/>
       <c r="B1" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
       <c r="F1" s="29"/>
-      <c r="G1" s="56" t="s">
+      <c r="G1" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="57"/>
-      <c r="I1" s="57"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
+      <c r="H1" s="85"/>
+      <c r="I1" s="85"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="85"/>
+      <c r="L1" s="85"/>
     </row>
     <row r="2" spans="1:15" ht="13.5" customHeight="1" thickBot="1">
       <c r="B2" s="5"/>
@@ -1751,61 +1751,61 @@
       <c r="F3" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="58" t="s">
-        <v>109</v>
-      </c>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="58"/>
-      <c r="L3" s="58"/>
+      <c r="G3" s="86" t="s">
+        <v>107</v>
+      </c>
+      <c r="H3" s="86"/>
+      <c r="I3" s="86"/>
+      <c r="J3" s="86"/>
+      <c r="K3" s="86"/>
+      <c r="L3" s="86"/>
     </row>
     <row r="4" spans="1:15" ht="15.75" thickBot="1">
       <c r="A4" s="17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C4" s="38" t="s">
         <v>33</v>
       </c>
       <c r="D4" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="38" t="s">
-        <v>38</v>
-      </c>
       <c r="F4" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="G4" s="59" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="87" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="60"/>
-      <c r="I4" s="60"/>
-      <c r="J4" s="60"/>
-      <c r="K4" s="60"/>
-      <c r="L4" s="61"/>
+      <c r="H4" s="88"/>
+      <c r="I4" s="88"/>
+      <c r="J4" s="88"/>
+      <c r="K4" s="88"/>
+      <c r="L4" s="89"/>
     </row>
     <row r="5" spans="1:15" ht="15.75" thickBot="1">
       <c r="A5" s="18" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="39" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C5" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="39" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="D5" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="E5" s="39" t="s">
-        <v>71</v>
-      </c>
-      <c r="F5" s="71" t="s">
-        <v>40</v>
+      <c r="F5" s="65" t="s">
+        <v>38</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="23" t="s">
@@ -1826,22 +1826,22 @@
     </row>
     <row r="6" spans="1:15" ht="15.75" thickBot="1">
       <c r="A6" s="19" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B6" s="39" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C6" s="39" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D6" s="39" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E6" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="72" t="s">
-        <v>59</v>
+      <c r="F6" s="66" t="s">
+        <v>57</v>
       </c>
       <c r="G6" s="30" t="s">
         <v>8</v>
@@ -1854,17 +1854,17 @@
     </row>
     <row r="7" spans="1:15" ht="15.75" thickBot="1">
       <c r="A7" s="20"/>
-      <c r="B7" s="73" t="s">
-        <v>68</v>
-      </c>
-      <c r="C7" s="74" t="s">
-        <v>45</v>
-      </c>
-      <c r="D7" s="74"/>
-      <c r="E7" s="74" t="s">
-        <v>72</v>
-      </c>
-      <c r="F7" s="83"/>
+      <c r="B7" s="67" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="68" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="68"/>
+      <c r="E7" s="68" t="s">
+        <v>70</v>
+      </c>
+      <c r="F7" s="77"/>
       <c r="G7" s="31" t="s">
         <v>15</v>
       </c>
@@ -1874,83 +1874,83 @@
       <c r="K7" s="14"/>
       <c r="L7" s="16"/>
     </row>
-    <row r="8" spans="1:15" ht="17.25" thickBot="1">
+    <row r="8" spans="1:15" ht="15.75" thickBot="1">
       <c r="A8" s="19" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B8" s="54" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C8" s="41" t="s">
+        <v>88</v>
+      </c>
+      <c r="D8" s="52" t="s">
         <v>90</v>
       </c>
-      <c r="D8" s="52" t="s">
+      <c r="E8" s="81" t="s">
         <v>92</v>
       </c>
-      <c r="E8" s="87" t="s">
-        <v>94</v>
-      </c>
       <c r="F8" s="37" t="s">
-        <v>104</v>
-      </c>
-      <c r="G8" s="58" t="s">
-        <v>110</v>
-      </c>
-      <c r="H8" s="58"/>
-      <c r="I8" s="58"/>
-      <c r="J8" s="58"/>
-      <c r="K8" s="58"/>
-      <c r="L8" s="58"/>
+        <v>102</v>
+      </c>
+      <c r="G8" s="86" t="s">
+        <v>108</v>
+      </c>
+      <c r="H8" s="86"/>
+      <c r="I8" s="86"/>
+      <c r="J8" s="86"/>
+      <c r="K8" s="86"/>
+      <c r="L8" s="86"/>
       <c r="N8" s="42"/>
     </row>
     <row r="9" spans="1:15" ht="15.75" thickBot="1">
       <c r="A9" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="76" t="s">
-        <v>73</v>
+      <c r="B9" s="70" t="s">
+        <v>71</v>
       </c>
       <c r="C9" s="39" t="s">
-        <v>108</v>
-      </c>
-      <c r="D9" s="77" t="s">
-        <v>63</v>
-      </c>
-      <c r="E9" s="76" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9" s="71" t="s">
-        <v>41</v>
-      </c>
-      <c r="G9" s="59" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="71" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" s="70" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" s="65" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="87" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="60"/>
-      <c r="I9" s="60"/>
-      <c r="J9" s="60"/>
-      <c r="K9" s="60"/>
-      <c r="L9" s="61"/>
+      <c r="H9" s="88"/>
+      <c r="I9" s="88"/>
+      <c r="J9" s="88"/>
+      <c r="K9" s="88"/>
+      <c r="L9" s="89"/>
       <c r="N9" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="15.75" thickBot="1">
       <c r="A10" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" s="77" t="s">
-        <v>75</v>
+        <v>52</v>
+      </c>
+      <c r="B10" s="71" t="s">
+        <v>73</v>
       </c>
       <c r="C10" s="39" t="s">
+        <v>89</v>
+      </c>
+      <c r="D10" s="69" t="s">
         <v>91</v>
       </c>
-      <c r="D10" s="75" t="s">
-        <v>93</v>
-      </c>
       <c r="E10" s="39" t="s">
-        <v>61</v>
-      </c>
-      <c r="F10" s="72"/>
+        <v>59</v>
+      </c>
+      <c r="F10" s="66"/>
       <c r="G10" s="11"/>
       <c r="H10" s="23" t="s">
         <v>9</v>
@@ -1971,18 +1971,18 @@
     <row r="11" spans="1:15" ht="15.75" thickBot="1">
       <c r="A11" s="20"/>
       <c r="B11" s="39" t="s">
-        <v>76</v>
-      </c>
-      <c r="C11" s="74" t="s">
-        <v>77</v>
-      </c>
-      <c r="D11" s="78" t="s">
-        <v>64</v>
-      </c>
-      <c r="E11" s="84" t="s">
-        <v>95</v>
-      </c>
-      <c r="F11" s="83"/>
+        <v>74</v>
+      </c>
+      <c r="C11" s="68" t="s">
+        <v>75</v>
+      </c>
+      <c r="D11" s="72" t="s">
+        <v>62</v>
+      </c>
+      <c r="E11" s="78" t="s">
+        <v>93</v>
+      </c>
+      <c r="F11" s="77"/>
       <c r="G11" s="30" t="s">
         <v>8</v>
       </c>
@@ -1992,22 +1992,22 @@
       <c r="K11" s="10"/>
       <c r="L11" s="24"/>
     </row>
-    <row r="12" spans="1:15" ht="17.25" thickBot="1">
+    <row r="12" spans="1:15" ht="15.75" thickBot="1">
       <c r="A12" s="17" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C12" s="54"/>
-      <c r="D12" s="88" t="s">
+      <c r="D12" s="82" t="s">
+        <v>101</v>
+      </c>
+      <c r="E12" s="54" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12" s="37" t="s">
         <v>103</v>
-      </c>
-      <c r="E12" s="54" t="s">
-        <v>78</v>
-      </c>
-      <c r="F12" s="37" t="s">
-        <v>105</v>
       </c>
       <c r="G12" s="31" t="s">
         <v>15</v>
@@ -2023,69 +2023,69 @@
         <v>7</v>
       </c>
       <c r="B13" s="39" t="s">
-        <v>87</v>
-      </c>
-      <c r="C13" s="76" t="s">
-        <v>36</v>
+        <v>85</v>
+      </c>
+      <c r="C13" s="70" t="s">
+        <v>34</v>
       </c>
       <c r="D13" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="76" t="s">
-        <v>79</v>
-      </c>
-      <c r="F13" s="72" t="s">
-        <v>42</v>
-      </c>
-      <c r="G13" s="58" t="s">
-        <v>111</v>
-      </c>
-      <c r="H13" s="58"/>
-      <c r="I13" s="58"/>
-      <c r="J13" s="58"/>
-      <c r="K13" s="58"/>
-      <c r="L13" s="58"/>
-    </row>
-    <row r="14" spans="1:15" ht="17.25" thickBot="1">
+      <c r="E13" s="70" t="s">
+        <v>77</v>
+      </c>
+      <c r="F13" s="66" t="s">
+        <v>40</v>
+      </c>
+      <c r="G13" s="86" t="s">
+        <v>109</v>
+      </c>
+      <c r="H13" s="86"/>
+      <c r="I13" s="86"/>
+      <c r="J13" s="86"/>
+      <c r="K13" s="86"/>
+      <c r="L13" s="86"/>
+    </row>
+    <row r="14" spans="1:15" ht="15.75" thickBot="1">
       <c r="A14" s="19" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B14" s="39" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C14" s="39" t="s">
-        <v>101</v>
-      </c>
-      <c r="D14" s="79" t="s">
-        <v>52</v>
+        <v>99</v>
+      </c>
+      <c r="D14" s="73" t="s">
+        <v>50</v>
       </c>
       <c r="E14" s="39" t="s">
-        <v>80</v>
-      </c>
-      <c r="F14" s="72"/>
-      <c r="G14" s="59" t="s">
+        <v>78</v>
+      </c>
+      <c r="F14" s="66"/>
+      <c r="G14" s="87" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="60"/>
-      <c r="I14" s="60"/>
-      <c r="J14" s="60"/>
-      <c r="K14" s="60"/>
-      <c r="L14" s="61"/>
+      <c r="H14" s="88"/>
+      <c r="I14" s="88"/>
+      <c r="J14" s="88"/>
+      <c r="K14" s="88"/>
+      <c r="L14" s="89"/>
       <c r="O14" s="49"/>
     </row>
     <row r="15" spans="1:15" ht="15.75" thickBot="1">
       <c r="A15" s="18"/>
       <c r="B15" s="39" t="s">
-        <v>89</v>
-      </c>
-      <c r="C15" s="82" t="s">
-        <v>102</v>
-      </c>
-      <c r="D15" s="80" t="s">
-        <v>51</v>
-      </c>
-      <c r="E15" s="84"/>
-      <c r="F15" s="85"/>
+        <v>87</v>
+      </c>
+      <c r="C15" s="76" t="s">
+        <v>100</v>
+      </c>
+      <c r="D15" s="74" t="s">
+        <v>49</v>
+      </c>
+      <c r="E15" s="78"/>
+      <c r="F15" s="79"/>
       <c r="G15" s="11"/>
       <c r="H15" s="23" t="s">
         <v>9</v>
@@ -2104,23 +2104,23 @@
       </c>
       <c r="O15" s="12"/>
     </row>
-    <row r="16" spans="1:15" ht="17.25" thickBot="1">
-      <c r="A16" s="65" t="s">
-        <v>57</v>
-      </c>
-      <c r="B16" s="66" t="s">
-        <v>82</v>
-      </c>
-      <c r="C16" s="67" t="s">
-        <v>96</v>
-      </c>
-      <c r="D16" s="75" t="s">
-        <v>47</v>
-      </c>
-      <c r="E16" s="67" t="s">
-        <v>100</v>
-      </c>
-      <c r="F16" s="81" t="s">
+    <row r="16" spans="1:15" ht="15.75" thickBot="1">
+      <c r="A16" s="59" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="60" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="61" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" s="69" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" s="61" t="s">
+        <v>98</v>
+      </c>
+      <c r="F16" s="75" t="s">
         <v>32</v>
       </c>
       <c r="G16" s="30" t="s">
@@ -2138,18 +2138,18 @@
         <v>7</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C17" s="39" t="s">
-        <v>97</v>
-      </c>
-      <c r="D17" s="77" t="s">
-        <v>98</v>
+        <v>95</v>
+      </c>
+      <c r="D17" s="71" t="s">
+        <v>96</v>
       </c>
       <c r="E17" s="39" t="s">
-        <v>48</v>
-      </c>
-      <c r="F17" s="72" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="66" t="s">
         <v>31</v>
       </c>
       <c r="G17" s="31" t="s">
@@ -2164,57 +2164,57 @@
     </row>
     <row r="18" spans="1:15" ht="15.75" thickBot="1">
       <c r="A18" s="22" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B18" s="39" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C18" s="39" t="s">
-        <v>62</v>
-      </c>
-      <c r="D18" s="75" t="s">
-        <v>99</v>
+        <v>60</v>
+      </c>
+      <c r="D18" s="69" t="s">
+        <v>97</v>
       </c>
       <c r="E18" s="39" t="s">
-        <v>81</v>
-      </c>
-      <c r="F18" s="72" t="s">
-        <v>43</v>
-      </c>
-      <c r="G18" s="58" t="s">
-        <v>112</v>
-      </c>
-      <c r="H18" s="58"/>
-      <c r="I18" s="58"/>
-      <c r="J18" s="58"/>
-      <c r="K18" s="58"/>
-      <c r="L18" s="58"/>
+        <v>79</v>
+      </c>
+      <c r="F18" s="66" t="s">
+        <v>41</v>
+      </c>
+      <c r="G18" s="86" t="s">
+        <v>110</v>
+      </c>
+      <c r="H18" s="86"/>
+      <c r="I18" s="86"/>
+      <c r="J18" s="86"/>
+      <c r="K18" s="86"/>
+      <c r="L18" s="86"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" thickBot="1">
-      <c r="A19" s="68"/>
-      <c r="B19" s="73" t="s">
-        <v>85</v>
-      </c>
-      <c r="C19" s="74"/>
-      <c r="D19" s="78"/>
-      <c r="E19" s="74" t="s">
-        <v>49</v>
-      </c>
-      <c r="F19" s="86"/>
-      <c r="G19" s="59" t="s">
+      <c r="A19" s="62"/>
+      <c r="B19" s="67" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="68"/>
+      <c r="D19" s="72"/>
+      <c r="E19" s="68" t="s">
+        <v>47</v>
+      </c>
+      <c r="F19" s="80"/>
+      <c r="G19" s="87" t="s">
         <v>18</v>
       </c>
-      <c r="H19" s="60"/>
-      <c r="I19" s="60"/>
-      <c r="J19" s="60"/>
-      <c r="K19" s="60"/>
-      <c r="L19" s="61"/>
-    </row>
-    <row r="20" spans="1:15" ht="17.25" thickBot="1">
+      <c r="H19" s="88"/>
+      <c r="I19" s="88"/>
+      <c r="J19" s="88"/>
+      <c r="K19" s="88"/>
+      <c r="L19" s="89"/>
+    </row>
+    <row r="20" spans="1:15" ht="15.75" thickBot="1">
       <c r="A20" s="22"/>
       <c r="B20" s="12"/>
       <c r="C20" s="49"/>
-      <c r="D20" s="62"/>
+      <c r="D20" s="56"/>
       <c r="E20" s="12"/>
       <c r="F20" s="12"/>
       <c r="G20" s="11"/>
@@ -2234,13 +2234,13 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="22.5" thickBot="1">
+    <row r="21" spans="1:15" ht="18.75" thickBot="1">
       <c r="A21" s="21"/>
       <c r="B21" s="12"/>
-      <c r="C21" s="89" t="s">
-        <v>107</v>
-      </c>
-      <c r="D21" s="89"/>
+      <c r="C21" s="83" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="83"/>
       <c r="E21" s="12"/>
       <c r="F21" s="12"/>
       <c r="G21" s="30" t="s">
@@ -2261,7 +2261,7 @@
       <c r="C22" s="12"/>
       <c r="D22" s="12"/>
       <c r="E22" s="12"/>
-      <c r="F22" s="63"/>
+      <c r="F22" s="57"/>
       <c r="G22" s="31" t="s">
         <v>15</v>
       </c>
@@ -2274,16 +2274,16 @@
     <row r="23" spans="1:15">
       <c r="A23" s="55"/>
       <c r="B23" s="12"/>
-      <c r="C23" s="64"/>
-      <c r="D23" s="64"/>
+      <c r="C23" s="58"/>
+      <c r="D23" s="58"/>
       <c r="E23" s="12"/>
       <c r="F23" s="50"/>
-      <c r="G23" s="58"/>
-      <c r="H23" s="58"/>
-      <c r="I23" s="58"/>
-      <c r="J23" s="58"/>
-      <c r="K23" s="58"/>
-      <c r="L23" s="58"/>
+      <c r="G23" s="86"/>
+      <c r="H23" s="86"/>
+      <c r="I23" s="86"/>
+      <c r="J23" s="86"/>
+      <c r="K23" s="86"/>
+      <c r="L23" s="86"/>
     </row>
     <row r="24" spans="1:15">
       <c r="A24" s="3"/>
@@ -2292,16 +2292,16 @@
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
       <c r="F24" s="12"/>
-      <c r="G24" s="58"/>
-      <c r="H24" s="58"/>
-      <c r="I24" s="58"/>
-      <c r="J24" s="58"/>
-      <c r="K24" s="58"/>
-      <c r="L24" s="58"/>
+      <c r="G24" s="86"/>
+      <c r="H24" s="86"/>
+      <c r="I24" s="86"/>
+      <c r="J24" s="86"/>
+      <c r="K24" s="86"/>
+      <c r="L24" s="86"/>
     </row>
     <row r="25" spans="1:15" ht="18.75">
       <c r="A25" s="6" t="s">
-        <v>34</v>
+        <v>111</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -2319,7 +2319,7 @@
     </row>
     <row r="26" spans="1:15" ht="15.75">
       <c r="A26" s="6" t="s">
-        <v>35</v>
+        <v>112</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -2327,15 +2327,15 @@
       <c r="E26" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="F26" s="69"/>
+      <c r="F26" s="63"/>
       <c r="G26" s="12"/>
-      <c r="H26" s="70"/>
-      <c r="I26" s="70"/>
-      <c r="J26" s="70"/>
-      <c r="K26" s="70"/>
-      <c r="L26" s="70"/>
-    </row>
-    <row r="27" spans="1:15" ht="26.25">
+      <c r="H26" s="64"/>
+      <c r="I26" s="64"/>
+      <c r="J26" s="64"/>
+      <c r="K26" s="64"/>
+      <c r="L26" s="64"/>
+    </row>
+    <row r="27" spans="1:15" ht="23.25">
       <c r="A27" s="5"/>
       <c r="B27" s="25" t="s">
         <v>21</v>
@@ -2349,11 +2349,11 @@
       </c>
       <c r="F27" s="12"/>
       <c r="G27" s="12"/>
-      <c r="H27" s="70"/>
-      <c r="I27" s="70"/>
-      <c r="J27" s="70"/>
-      <c r="K27" s="70"/>
-      <c r="L27" s="70"/>
+      <c r="H27" s="64"/>
+      <c r="I27" s="64"/>
+      <c r="J27" s="64"/>
+      <c r="K27" s="64"/>
+      <c r="L27" s="64"/>
     </row>
     <row r="28" spans="1:15">
       <c r="A28" s="3"/>

</xml_diff>